<commit_message>
successful valid file ingestion completed
</commit_message>
<xml_diff>
--- a/tests/sample_artifacts/valid/excel/valid_customers_001.xlsx
+++ b/tests/sample_artifacts/valid/excel/valid_customers_001.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Customers_AU" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Customers_US" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Reference" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="d/mm/yyyy;@"/>
+    <numFmt numFmtId="167" formatCode="m/d/yyyy;@"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -48,8 +52,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,11 +457,6 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>DateLocaleTag</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
           <t>SourceSystem</t>
         </is>
       </c>
@@ -471,10 +472,8 @@
           <t>Customer 1100</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2024-01-08</t>
-        </is>
+      <c r="C2" s="1" t="n">
+        <v>45299</v>
       </c>
       <c r="D2" t="n">
         <v>1550</v>
@@ -491,11 +490,6 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[$-en-AU]</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -511,10 +505,8 @@
           <t>Customer 1101</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2024-01-09</t>
-        </is>
+      <c r="C3" s="1" t="n">
+        <v>45300</v>
       </c>
       <c r="D3" t="n">
         <v>1585.75</v>
@@ -531,11 +523,6 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[$-en-AU]</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -551,10 +538,8 @@
           <t>Customer 1102</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2024-01-10</t>
-        </is>
+      <c r="C4" s="1" t="n">
+        <v>45301</v>
       </c>
       <c r="D4" t="n">
         <v>1621.5</v>
@@ -571,11 +556,6 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>[$-en-AU]</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -591,10 +571,8 @@
           <t>Customer 1103</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2024-01-11</t>
-        </is>
+      <c r="C5" s="1" t="n">
+        <v>45302</v>
       </c>
       <c r="D5" t="n">
         <v>1657.25</v>
@@ -611,11 +589,6 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>[$-en-AU]</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -631,10 +604,8 @@
           <t>Customer 1104</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2024-01-12</t>
-        </is>
+      <c r="C6" s="1" t="n">
+        <v>45303</v>
       </c>
       <c r="D6" t="n">
         <v>1693</v>
@@ -651,11 +622,6 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>[$-en-AU]</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -671,10 +637,8 @@
           <t>Customer 1105</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2024-01-13</t>
-        </is>
+      <c r="C7" s="1" t="n">
+        <v>45304</v>
       </c>
       <c r="D7" t="n">
         <v>1728.75</v>
@@ -691,11 +655,6 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>[$-en-AU]</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -711,10 +670,8 @@
           <t>Customer 1106</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2024-01-14</t>
-        </is>
+      <c r="C8" s="1" t="n">
+        <v>45305</v>
       </c>
       <c r="D8" t="n">
         <v>1764.5</v>
@@ -731,11 +688,6 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>[$-en-AU]</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -751,10 +703,8 @@
           <t>Customer 1107</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2024-01-15</t>
-        </is>
+      <c r="C9" s="1" t="n">
+        <v>45306</v>
       </c>
       <c r="D9" t="n">
         <v>1800.25</v>
@@ -770,11 +720,6 @@
         </is>
       </c>
       <c r="G9" t="inlineStr">
-        <is>
-          <t>[$-en-AU]</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
         <is>
           <t>CRM</t>
         </is>
@@ -791,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -827,11 +772,6 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>DateLocaleTag</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
           <t>SourceSystem</t>
         </is>
       </c>
@@ -847,10 +787,8 @@
           <t>Customer 2100</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2024-01-08</t>
-        </is>
+      <c r="C2" s="2" t="n">
+        <v>45299</v>
       </c>
       <c r="D2" t="n">
         <v>1550</v>
@@ -867,11 +805,6 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[$-en-US]</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -887,10 +820,8 @@
           <t>Customer 2101</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2024-01-09</t>
-        </is>
+      <c r="C3" s="2" t="n">
+        <v>45300</v>
       </c>
       <c r="D3" t="n">
         <v>1585.75</v>
@@ -907,11 +838,6 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[$-en-US]</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -927,10 +853,8 @@
           <t>Customer 2102</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2024-01-10</t>
-        </is>
+      <c r="C4" s="2" t="n">
+        <v>45301</v>
       </c>
       <c r="D4" t="n">
         <v>1621.5</v>
@@ -947,11 +871,6 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>[$-en-US]</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -967,10 +886,8 @@
           <t>Customer 2103</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2024-01-11</t>
-        </is>
+      <c r="C5" s="2" t="n">
+        <v>45302</v>
       </c>
       <c r="D5" t="n">
         <v>1657.25</v>
@@ -987,11 +904,6 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>[$-en-US]</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -1007,10 +919,8 @@
           <t>Customer 2104</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2024-01-12</t>
-        </is>
+      <c r="C6" s="2" t="n">
+        <v>45303</v>
       </c>
       <c r="D6" t="n">
         <v>1693</v>
@@ -1027,11 +937,6 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>[$-en-US]</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -1047,10 +952,8 @@
           <t>Customer 2105</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2024-01-13</t>
-        </is>
+      <c r="C7" s="2" t="n">
+        <v>45304</v>
       </c>
       <c r="D7" t="n">
         <v>1728.75</v>
@@ -1067,11 +970,6 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>[$-en-US]</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -1087,10 +985,8 @@
           <t>Customer 2106</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2024-01-14</t>
-        </is>
+      <c r="C8" s="2" t="n">
+        <v>45305</v>
       </c>
       <c r="D8" t="n">
         <v>1764.5</v>
@@ -1107,11 +1003,6 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>[$-en-US]</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
           <t>CRM</t>
         </is>
       </c>
@@ -1127,10 +1018,8 @@
           <t>Customer 2107</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2024-01-15</t>
-        </is>
+      <c r="C9" s="2" t="n">
+        <v>45306</v>
       </c>
       <c r="D9" t="n">
         <v>1800.25</v>
@@ -1147,77 +1036,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>[$-en-US]</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>CRM</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>RegionCode</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>RegionName</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>CurrencyCode</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>AU</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>USD</t>
+          <t>CRM</t>
         </is>
       </c>
     </row>

</xml_diff>